<commit_message>
Regenerate test-data Excel files for admin and faculty workflows.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/test-data/faculty.xlsx
+++ b/test-data/faculty.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Faculty" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,7 +446,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0501112233</t>
+          <t>0551111111</t>
         </is>
       </c>
     </row>
@@ -463,7 +463,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0504445566</t>
+          <t>0552222222</t>
         </is>
       </c>
     </row>

</xml_diff>